<commit_message>
Added in some documents
</commit_message>
<xml_diff>
--- a/app/static/templates/EAD.xlsx
+++ b/app/static/templates/EAD.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +29,85 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001e293b"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3C5E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F7FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E8F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -42,12 +115,131 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001A3C5E"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -410,70 +602,1302 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="009333EA"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Loan ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Customer ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>SEGMENT</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Reporting Date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Maturity Date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Adjusted Maturity Date</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>First Payment Date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Outstanding Amount</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Repayment Frequency</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Effective Interest Rate (EIR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LN-2025-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2029-03-31</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>2029-03-31</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>2022-04-30</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>490000</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>LN-2025-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>2028-06-30</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>2028-06-30</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>2021-07-31</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>748000</v>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>LN-2025-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CUST-002</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2030-12-31</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2030-12-31</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>LN-2025-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>CUST-003</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>2023-10-31</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>1060000</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>LN-2025-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>CUST-003</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>2027-03-31</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2027-03-31</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2022-04-30</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>860000</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>LN-2025-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>CUST-004</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>2031-03-31</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>2031-03-31</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>2024-04-30</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>LN-2025-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CUST-005</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2023-04-30</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>425000</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>LN-2025-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>CUST-005</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>2028-09-30</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>2028-09-30</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>2022-10-31</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>980000</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LN-2025-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CUST-006</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>2032-06-30</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2032-06-30</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>2024-07-31</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>LN-2025-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>CUST-007</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>SME</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>2027-09-30</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>2027-09-30</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>2023-10-31</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>630000</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="I2:I50000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose from the list: Repayment Frequency" promptTitle="Repayment Frequency" prompt="MTH = Monthly  |  QTR = Quarterly" type="list">
+      <formula1>"MTH,QTR"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J50000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose from the list: Staging" promptTitle="Staging" prompt="Stage 1 = performing  |  Stage 2 = SICR  |  Stage 3 = default" type="list">
+      <formula1>"Stage 1,Stage 2,Stage 3"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="009333EA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Exposure at Default (EAD) — Upload Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Upload one EAD file per run (single workbook, 25 MB max).  Each row is one active loan at the reporting date.  The engine performs a month-by-month forward balance walk (up to 299 months) computing the expected outstanding balance at each future period, then discounts the resulting ECL cash flows back to today.</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="13" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Column Name</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Allowed Values</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Business Rule</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Loan ID</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Unique, non-empty</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Must be unique within this file.  Primary key for the EAD rundown and for joining PD and LGD results at the loan level.</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>LN-2025-0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Customer ID</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Non-empty string</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>Used to join LGD collateral data.  Must match the Customer ID in the LGD file.</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>SEGMENT</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Must match a configured segment</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Case-sensitive match to a Segment name in Workspace → Admin → Segments.  Used to look up the segment-level PD curve.</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Reporting Date</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>The as-at snapshot date for this loan.  All other dates are validated relative to this.</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Maturity Date</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>≥ Reporting Date</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Contractual maturity date.  Must be on or after Reporting Date (EC-03).  The rundown stops at this date.</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>2029-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Adjusted Maturity Date</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>≥ First Payment Date</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>Effective maturity after any restructuring or extensions.  Must be on or after First Payment Date.</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>2029-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>First Payment Date</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>≤ Reporting Date</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Date of the first scheduled repayment.  Must be on or before Reporting Date (EC-04).  Used to determine remaining loan term.</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>2022-04-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Outstanding Amount</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>≥ 0</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Current outstanding principal balance at the reporting date.  Seed value for the forward balance walk.</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>490000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Repayment Frequency</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Enum</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>MTH  or  QTR</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Payment schedule frequency.  MTH = monthly, QTR = quarterly.  Other values trigger EC-09.  The balance walk always accrues monthly regardless.</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Enum</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Stage 1  /  Stage 2  /  Stage 3</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>IFRS 9 credit stage at the reporting date.  Determines which row of the segment PD transition matrix is used for lifetime marginal PD.</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Effective Interest Rate (EIR)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Repayment Frequency</t>
-        </is>
-      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>0 – 1  (decimal fraction)</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Annual EIR as a decimal, e.g. 0.14 for 14 %.  Used for (a) instalment calculation and (b) ECL discounting (EC-05: must be in the range 0 – 1).</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>0.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Cross-field date validation rules  (violations block the run)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>EC-03   Maturity Date  ≥  Reporting Date</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="13" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ✗  Reporting Date = 2025-03-31,  Maturity Date = 2024-12-31   ← maturity is in the past</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ✓  Reporting Date = 2025-03-31,  Maturity Date = 2029-03-31</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="13" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="17" t="inlineStr"/>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="13" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>EC-04   First Payment Date  ≤  Reporting Date</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="13" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ✗  Reporting Date = 2025-03-31,  First Payment Date = 2025-06-30   ← first payment in the future</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="13" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ✓  Reporting Date = 2025-03-31,  First Payment Date = 2022-04-30</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="13" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="17" t="inlineStr"/>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="13" t="n"/>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Adjusted Maturity Date  ≥  First Payment Date</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="13" t="n"/>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ✗  First Payment Date = 2022-04-30,  Adjusted Maturity Date = 2021-12-31</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="13" t="n"/>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ✓  First Payment Date = 2022-04-30,  Adjusted Maturity Date = 2029-03-31</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="13" t="n"/>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Balance walk and instalment calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>For MTH loans:  monthly instalment = PMT(EIR / 12, remaining_months, outstanding)</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="13" t="n"/>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>For QTR loans:  quarterly instalment = PMT(EIR / 4,  remaining_quarters, outstanding)</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="13" t="n"/>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Monthly balance accrual always uses  EIR / 12  regardless of payment frequency.</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="13" t="n"/>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Stage 3 loans accrue missed-payment interest into the balance at each forward step.</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n"/>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="13" t="n"/>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>The rundown produces up to 299 monthly EAD snapshots per loan.</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="13" t="n"/>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Accepted aliases for column names</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Staging column also accepted as:   Staging (Stage)</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n"/>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="13" t="n"/>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>EIR column also accepted as:       Effective Interest Rate   or   EIR</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="13" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>